<commit_message>
human rating is added to input and output files
</commit_message>
<xml_diff>
--- a/RelevanceIQ_Input_Data_Schema.xlsx
+++ b/RelevanceIQ_Input_Data_Schema.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vs code\RelevanceIQ  - FTO - FSP - Cache - Copy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vs code\New\RelevanceIQ  - FTO - html_css-file - Copy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD6DC7F-DC9E-4C71-A5DB-7EAE4B870977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D68316-7665-4655-9508-6528D265DEE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E4A06896-3B68-432A-A172-83E6F9A49BE2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Abstract</t>
   </si>
@@ -40,6 +40,9 @@
   </si>
   <si>
     <t>Title</t>
+  </si>
+  <si>
+    <t>Relevance Human</t>
   </si>
 </sst>
 </file>
@@ -537,7 +540,9 @@
       <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="6"/>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>

</xml_diff>